<commit_message>
Dyed waivers: Idaho ends Nov 7, North Carolina runs Oct 9 to Dec 31
Idaho's order runs thirty calendar days from Oct 9 unless a later order rescinds or extends it. North Carolina's dates are now its penalty relief; the zero-tax weeks are in the note.
</commit_message>
<xml_diff>
--- a/General/Dyed waivers/Dyed Waivers.xlsx
+++ b/General/Dyed waivers/Dyed Waivers.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AECD9F3-DD99-48F0-9543-B013BD7391AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA69FBB3-129A-4C7C-9851-59DD95C227CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dyed diesel" sheetId="1" r:id="rId1"/>
@@ -166,7 +166,7 @@
     <t>Idaho</t>
   </si>
   <si>
-    <t>Executive Order 2026-07, signed Oct 9, 2026; thirty calendar days unless rescinded or extended, so to about Nov 7 or 8</t>
+    <t>Executive Order 2026-07, signed Oct 9, 2026; it stays in effect thirty calendar days unless a later order of the Governor rescinds or extends it. Day one is Oct 9, the day it was signed, so day thirty is Nov 7.</t>
   </si>
   <si>
     <t>Illinois</t>
@@ -256,7 +256,7 @@
     <t>North Carolina</t>
   </si>
   <si>
-    <t>Session Law 2026-62 (House Bill 3), approved Oct 9, 2026; the Department of Revenue Important Notice of Oct 12, 2026, which overrides earlier guidance where they conflict. The dates are the weeks the tax is zero; no state penalty on farm use, or on whoever dispenses the dyed, Oct 9 through Dec 31</t>
+    <t>Session Law 2026-62 (House Bill 3), approved Oct 9, 2026; the Department of Revenue Important Notice of Oct 12, 2026, which overrides earlier guidance where they conflict. The dates are the penalty relief, for farm use or whoever dispenses the dyed. The tax is zero for everyone only Oct 10 to Nov 30; a holder of a Department exemption certificate owes none Oct 1 to Dec 31.</t>
   </si>
   <si>
     <t>North Dakota</t>
@@ -1141,13 +1141,13 @@
         <v>46310</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B14" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>In effect, no end date</v>
+        <v>In effect</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>23</v>
@@ -1161,12 +1161,14 @@
       <c r="F14" s="11">
         <v>46304</v>
       </c>
-      <c r="G14" s="11"/>
+      <c r="G14" s="11">
+        <v>46333</v>
+      </c>
       <c r="H14" s="10" t="s">
         <v>43</v>
       </c>
       <c r="I14" s="11">
-        <v>46308</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1549,7 +1551,7 @@
         <v>46308</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>72</v>
       </c>
@@ -1567,10 +1569,10 @@
         <v>20</v>
       </c>
       <c r="F28" s="11">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="G28" s="11">
-        <v>46356</v>
+        <v>46387</v>
       </c>
       <c r="H28" s="10" t="s">
         <v>73</v>

</xml_diff>